<commit_message>
Dados atualizados via Robô: 18/05/2026 17:40
</commit_message>
<xml_diff>
--- a/sipii_caixa_20260518.xlsx
+++ b/sipii_caixa_20260518.xlsx
@@ -581,7 +581,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>408,551</t>
+          <t>406,838</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -603,7 +603,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF FÁCIL RF SIMPLES RESP LTDA</t>
+          <t>CAIXA FIC FIF FÁCIL RF SIMPLES RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -638,7 +638,7 @@
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>6.726,533</t>
+          <t>6.646,913</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
@@ -660,7 +660,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF MOVIMENTAÇÕES AUTOMÁTICAS RF SIMPLES RESP LTDA</t>
+          <t>CAIXA FIC FIF MOVIMENTAÇÕES AUTOMÁTICAS RF SIMPLES RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -695,7 +695,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>810,624</t>
+          <t>810,007</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -809,7 +809,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>120,092</t>
+          <t>120,091</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -866,7 +866,7 @@
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>96,153</t>
+          <t>96,136</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
@@ -923,7 +923,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>584,603</t>
+          <t>584,596</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -980,7 +980,7 @@
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>61,658</t>
+          <t>61,657</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>1.672,750</t>
+          <t>1.672,699</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -1147,7 +1147,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>28,420</t>
+          <t>28,419</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1318,7 +1318,7 @@
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>79,712</t>
+          <t>79,693</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
@@ -1489,7 +1489,7 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>140,753</t>
+          <t>140,752</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
@@ -1546,7 +1546,7 @@
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>1.756,434</t>
+          <t>1.740,789</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
@@ -1603,7 +1603,7 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>2.192,986</t>
+          <t>2.192,972</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -1774,7 +1774,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>957,119</t>
+          <t>957,109</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -1796,7 +1796,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>CAIXA EXPERT ARX IPCA DEB INCENTIVADAS FIC FIF RF CRED PRIV - RESP LTDA (1) (2)</t>
+          <t>CAIXA EXPERT ARX IPCA DEB INCENTIVADAS FIC FIF RF CRED PRIV - RESP LTDA (2)</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -1806,32 +1806,32 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,10997325</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>-0,001</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>0,00</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>2,89</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>219,622</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
@@ -1853,7 +1853,7 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIF FIC EXPERT SULAMERICA RF CRED PRIV LP - RESP LTDA (1)</t>
+          <t>CAIXA FIF FIC EXPERT SULAMERICA RF CRED PRIV LP - RESP LTDA</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
@@ -1863,32 +1863,32 @@
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F25" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H25" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,22811400</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>-0,001</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>0,62</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>4,85</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>14,63</t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>70,980</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
@@ -1945,7 +1945,7 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>175,319</t>
+          <t>175,223</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
@@ -2024,7 +2024,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>CAIXA EXPERT VOX DESENV SUSTENTAVEL IS RF CRED PRIV LP - RESP LTDA (1) (2)</t>
+          <t>CAIXA EXPERT VOX DESENV SUSTENTAVEL IS RF CRED PRIV LP - RESP LTDA (2)</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -2034,32 +2034,32 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,02936900</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>-0,001</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>0,52</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>4,97</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>21,758</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
@@ -2077,7 +2077,7 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>CAIXA EXPERT ABSOLUTE CRETA FIC FIF RF CRED PRIV LP - RESP LTDA (1)</t>
+          <t>CAIXA EXPERT ABSOLUTE CRETA FIC FIF RF CRED PRIV LP - RESP LTDA</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
@@ -2087,32 +2087,32 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H29" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,15576700</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>-0,001</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>0,66</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>4,08</t>
+        </is>
+      </c>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>13,73</t>
         </is>
       </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>66,353</t>
         </is>
       </c>
       <c r="J29" s="4" t="inlineStr">
@@ -2130,7 +2130,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>CAIXA EXPERT RB ASSET CDI DEB INCENTIVADAS FIC FIF RF CRED PRIV RESP LTDA (1) (2)</t>
+          <t>CAIXA EXPERT RB ASSET CDI DEB INCENTIVADAS FIC FIF RF CRED PRIV RESP LTDA (2)</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -2140,32 +2140,32 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,05776364</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>-0,001</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>0,31</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>2,36</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>332,405</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
@@ -2187,7 +2187,7 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>CAIXA EXPERT VINLAND DEB IN INFRA RF CRED PRIV LP RESP LTDA (1) (2) (3)</t>
+          <t>CAIXA EXPERT VINLAND DEB IN INFRA RF CRED PRIV LP RESP LTDA (2) (3)</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
@@ -2275,7 +2275,7 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>859,898</t>
+          <t>859,833</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
@@ -2332,7 +2332,7 @@
       </c>
       <c r="I33" s="4" t="inlineStr">
         <is>
-          <t>3.241,411</t>
+          <t>3.241,339</t>
         </is>
       </c>
       <c r="J33" s="4" t="inlineStr">
@@ -2446,7 +2446,7 @@
       </c>
       <c r="I35" s="4" t="inlineStr">
         <is>
-          <t>3.113,953</t>
+          <t>3.113,942</t>
         </is>
       </c>
       <c r="J35" s="4" t="inlineStr">
@@ -2503,7 +2503,7 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>125,145</t>
+          <t>125,015</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
@@ -2560,7 +2560,7 @@
       </c>
       <c r="I37" s="4" t="inlineStr">
         <is>
-          <t>550,004</t>
+          <t>549,999</t>
         </is>
       </c>
       <c r="J37" s="4" t="inlineStr">
@@ -2674,7 +2674,7 @@
       </c>
       <c r="I39" s="4" t="inlineStr">
         <is>
-          <t>334,888</t>
+          <t>334,883</t>
         </is>
       </c>
       <c r="J39" s="4" t="inlineStr">
@@ -2731,7 +2731,7 @@
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>2.373,675</t>
+          <t>2.373,657</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
@@ -2788,7 +2788,7 @@
       </c>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>553,400</t>
+          <t>553,399</t>
         </is>
       </c>
       <c r="J41" s="4" t="inlineStr">
@@ -2845,7 +2845,7 @@
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>15.485,298</t>
+          <t>15.485,082</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -2902,7 +2902,7 @@
       </c>
       <c r="I43" s="4" t="inlineStr">
         <is>
-          <t>1.383,497</t>
+          <t>1.383,496</t>
         </is>
       </c>
       <c r="J43" s="4" t="inlineStr">
@@ -2959,7 +2959,7 @@
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>165,472</t>
+          <t>165,470</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
@@ -3069,7 +3069,7 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>6.013,909</t>
+          <t>5.952,431</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
@@ -3126,7 +3126,7 @@
       </c>
       <c r="I47" s="4" t="inlineStr">
         <is>
-          <t>2.188,952</t>
+          <t>2.188,909</t>
         </is>
       </c>
       <c r="J47" s="4" t="inlineStr">
@@ -3240,7 +3240,7 @@
       </c>
       <c r="I49" s="4" t="inlineStr">
         <is>
-          <t>839,422</t>
+          <t>839,413</t>
         </is>
       </c>
       <c r="J49" s="4" t="inlineStr">
@@ -3297,7 +3297,7 @@
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>15.546,151</t>
+          <t>15.545,914</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
@@ -3354,7 +3354,7 @@
       </c>
       <c r="I51" s="4" t="inlineStr">
         <is>
-          <t>9.466,109</t>
+          <t>9.466,015</t>
         </is>
       </c>
       <c r="J51" s="4" t="inlineStr">
@@ -3411,7 +3411,7 @@
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>20.846,276</t>
+          <t>20.845,858</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr">
@@ -3468,7 +3468,7 @@
       </c>
       <c r="I53" s="4" t="inlineStr">
         <is>
-          <t>13.169,981</t>
+          <t>13.169,776</t>
         </is>
       </c>
       <c r="J53" s="4" t="inlineStr">
@@ -3490,7 +3490,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF RENDA FIXA CURTO PRAZO RESP LTDA</t>
+          <t>CAIXA FIC FIF RENDA FIXA CURTO PRAZO RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -3525,7 +3525,7 @@
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>245,548</t>
+          <t>245,520</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr">
@@ -3547,7 +3547,7 @@
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF FOF SMART CRED PRIV MM LP RESP LTDA (1)</t>
+          <t>CAIXA FIC FIF FOF SMART CRED PRIV MM LP RESP LTDA</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
@@ -3557,32 +3557,32 @@
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E55" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F55" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G55" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H55" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,39931700</t>
+        </is>
+      </c>
+      <c r="E55" s="6" t="inlineStr">
+        <is>
+          <t>-0,007</t>
+        </is>
+      </c>
+      <c r="F55" s="5" t="inlineStr">
+        <is>
+          <t>0,60</t>
+        </is>
+      </c>
+      <c r="G55" s="5" t="inlineStr">
+        <is>
+          <t>4,51</t>
+        </is>
+      </c>
+      <c r="H55" s="5" t="inlineStr">
+        <is>
+          <t>14,12</t>
         </is>
       </c>
       <c r="I55" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>68,862</t>
         </is>
       </c>
       <c r="J55" s="4" t="inlineStr">
@@ -3604,7 +3604,7 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC MULTIGESTOR GLOBAL EQUITIES IE (1)</t>
+          <t>CAIXA FIC MULTIGESTOR GLOBAL EQUITIES IE</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -3614,32 +3614,32 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E56" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F56" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G56" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H56" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1.167,25373800</t>
+        </is>
+      </c>
+      <c r="E56" s="7" t="inlineStr">
+        <is>
+          <t>-0,003</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>1,55</t>
+        </is>
+      </c>
+      <c r="G56" s="7" t="inlineStr">
+        <is>
+          <t>-6,97</t>
+        </is>
+      </c>
+      <c r="H56" s="7" t="inlineStr">
+        <is>
+          <t>-2,47</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>35,739</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr">
@@ -3696,7 +3696,7 @@
       </c>
       <c r="I57" s="4" t="inlineStr">
         <is>
-          <t>328,493</t>
+          <t>540,035</t>
         </is>
       </c>
       <c r="J57" s="4" t="inlineStr">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF ESTRATÉGIA LIVRE MULTIMERCADO LP RESP LTDA (1)</t>
+          <t>CAIXA FIC FIF ESTRATÉGIA LIVRE MULTIMERCADO LP RESP LTDA</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -3728,32 +3728,32 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E58" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F58" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G58" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H58" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1.632,15053600</t>
+        </is>
+      </c>
+      <c r="E58" s="7" t="inlineStr">
+        <is>
+          <t>-0,006</t>
+        </is>
+      </c>
+      <c r="F58" s="7" t="inlineStr">
+        <is>
+          <t>-0,22</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="inlineStr">
+        <is>
+          <t>4,16</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr">
+        <is>
+          <t>13,39</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>116,889</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
@@ -3810,7 +3810,7 @@
       </c>
       <c r="I59" s="4" t="inlineStr">
         <is>
-          <t>13,423</t>
+          <t>13,348</t>
         </is>
       </c>
       <c r="J59" s="4" t="inlineStr">
@@ -3832,7 +3832,7 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>CAIXA CARTEIRA QUANT DUO FIC FIF MM LP RESP LTDA (1) (2) (3)</t>
+          <t>CAIXA CARTEIRA QUANT DUO FIC FIF MM LP RESP LTDA (2) (3)</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -3885,7 +3885,7 @@
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF FOF SMART LONG SHORT LP RESP LTDA (1)</t>
+          <t>CAIXA FIC FIF FOF SMART LONG SHORT LP RESP LTDA</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
@@ -3895,32 +3895,32 @@
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E61" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F61" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G61" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H61" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,25018500</t>
+        </is>
+      </c>
+      <c r="E61" s="6" t="inlineStr">
+        <is>
+          <t>-0,005</t>
+        </is>
+      </c>
+      <c r="F61" s="6" t="inlineStr">
+        <is>
+          <t>-0,44</t>
+        </is>
+      </c>
+      <c r="G61" s="5" t="inlineStr">
+        <is>
+          <t>2,36</t>
+        </is>
+      </c>
+      <c r="H61" s="5" t="inlineStr">
+        <is>
+          <t>11,60</t>
         </is>
       </c>
       <c r="I61" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>6,666</t>
         </is>
       </c>
       <c r="J61" s="4" t="inlineStr">
@@ -3999,7 +3999,7 @@
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>CAIXA CARTEIRA QUANT QUALI FIC FIF MM LP RESP LTDA (1) (2) (3)</t>
+          <t>CAIXA CARTEIRA QUANT QUALI FIC FIF MM LP RESP LTDA (2) (3)</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
@@ -4052,7 +4052,7 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF FOF SMART LONG BIAS MM RESP LTDA (1)</t>
+          <t>CAIXA FIC FIF FOF SMART LONG BIAS MM RESP LTDA</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -4062,32 +4062,32 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E64" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F64" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G64" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H64" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,44320300</t>
+        </is>
+      </c>
+      <c r="E64" s="7" t="inlineStr">
+        <is>
+          <t>-0,004</t>
+        </is>
+      </c>
+      <c r="F64" s="7" t="inlineStr">
+        <is>
+          <t>-1,73</t>
+        </is>
+      </c>
+      <c r="G64" s="3" t="inlineStr">
+        <is>
+          <t>5,72</t>
+        </is>
+      </c>
+      <c r="H64" s="3" t="inlineStr">
+        <is>
+          <t>21,08</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>11,970</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
@@ -4109,7 +4109,7 @@
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>CAIXA CARTEIRA QUANT UNO FIC FIF MM LP RESP LTDA (1) (2) (3)</t>
+          <t>CAIXA CARTEIRA QUANT UNO FIC FIF MM LP RESP LTDA (2) (3)</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
@@ -4219,7 +4219,7 @@
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF ESTRATÉGICO MULTIMERCADO LP RESP LTDA (1)</t>
+          <t>CAIXA FIC FIF ESTRATÉGICO MULTIMERCADO LP RESP LTDA</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
@@ -4229,32 +4229,32 @@
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E67" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F67" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G67" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H67" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>5,32047778</t>
+        </is>
+      </c>
+      <c r="E67" s="6" t="inlineStr">
+        <is>
+          <t>-0,003</t>
+        </is>
+      </c>
+      <c r="F67" s="6" t="inlineStr">
+        <is>
+          <t>-0,21</t>
+        </is>
+      </c>
+      <c r="G67" s="5" t="inlineStr">
+        <is>
+          <t>3,69</t>
+        </is>
+      </c>
+      <c r="H67" s="5" t="inlineStr">
+        <is>
+          <t>13,12</t>
         </is>
       </c>
       <c r="I67" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>33,192</t>
         </is>
       </c>
       <c r="J67" s="4" t="inlineStr">
@@ -4311,7 +4311,7 @@
       </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>668,164</t>
+          <t>666,467</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr">
@@ -4333,7 +4333,7 @@
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF FOF SMART MULTIESTRATEGIA MM RESP LTDA (1)</t>
+          <t>CAIXA FIC FIF FOF SMART MULTIESTRATEGIA MM RESP LTDA</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
@@ -4343,32 +4343,32 @@
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E69" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F69" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G69" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H69" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>2,85531700</t>
+        </is>
+      </c>
+      <c r="E69" s="6" t="inlineStr">
+        <is>
+          <t>-0,004</t>
+        </is>
+      </c>
+      <c r="F69" s="5" t="inlineStr">
+        <is>
+          <t>0,08</t>
+        </is>
+      </c>
+      <c r="G69" s="5" t="inlineStr">
+        <is>
+          <t>2,22</t>
+        </is>
+      </c>
+      <c r="H69" s="5" t="inlineStr">
+        <is>
+          <t>11,44</t>
         </is>
       </c>
       <c r="I69" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>77,229</t>
         </is>
       </c>
       <c r="J69" s="4" t="inlineStr">
@@ -4482,7 +4482,7 @@
       </c>
       <c r="I71" s="4" t="inlineStr">
         <is>
-          <t>2.330,280</t>
+          <t>2.329,776</t>
         </is>
       </c>
       <c r="J71" s="4" t="inlineStr">
@@ -4561,7 +4561,7 @@
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF FUNCIONARIOS ESTRATEGIA LIVRE MULTIMERCADO LP RESP LTDA (1)</t>
+          <t>CAIXA FIC FIF FUNCIONARIOS ESTRATEGIA LIVRE MULTIMERCADO LP RESP LTDA</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
@@ -4571,32 +4571,32 @@
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E73" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F73" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G73" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H73" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1.652,59401600</t>
+        </is>
+      </c>
+      <c r="E73" s="6" t="inlineStr">
+        <is>
+          <t>-0,003</t>
+        </is>
+      </c>
+      <c r="F73" s="6" t="inlineStr">
+        <is>
+          <t>-0,18</t>
+        </is>
+      </c>
+      <c r="G73" s="5" t="inlineStr">
+        <is>
+          <t>4,49</t>
+        </is>
+      </c>
+      <c r="H73" s="5" t="inlineStr">
+        <is>
+          <t>14,36</t>
         </is>
       </c>
       <c r="I73" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>15,317</t>
         </is>
       </c>
       <c r="J73" s="4" t="inlineStr">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>CAIXA HASHDEX NASDAQ CRYPTO INDEX FIC FIF MM RESP LTDA (1) (2)</t>
+          <t>CAIXA HASHDEX NASDAQ CRYPTO INDEX FIC FIF MM RESP LTDA (2)</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
@@ -4624,32 +4624,32 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E74" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F74" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G74" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>0,57593472</t>
+        </is>
+      </c>
+      <c r="E74" s="7" t="inlineStr">
+        <is>
+          <t>-0,007</t>
+        </is>
+      </c>
+      <c r="F74" s="3" t="inlineStr">
+        <is>
+          <t>6,16</t>
+        </is>
+      </c>
+      <c r="G74" s="7" t="inlineStr">
+        <is>
+          <t>-20,24</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0,00</t>
         </is>
       </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4,200</t>
         </is>
       </c>
       <c r="J74" s="2" t="inlineStr">
@@ -4667,7 +4667,7 @@
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF CAPITAL PROTEGIDO CESTA AGRO MM (1)</t>
+          <t>CAIXA FIC FIF CAPITAL PROTEGIDO CESTA AGRO MM</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
@@ -4677,32 +4677,32 @@
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E75" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F75" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G75" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H75" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,37874300</t>
+        </is>
+      </c>
+      <c r="E75" s="6" t="inlineStr">
+        <is>
+          <t>-0,003</t>
+        </is>
+      </c>
+      <c r="F75" s="6" t="inlineStr">
+        <is>
+          <t>-1,35</t>
+        </is>
+      </c>
+      <c r="G75" s="5" t="inlineStr">
+        <is>
+          <t>1,66</t>
+        </is>
+      </c>
+      <c r="H75" s="5" t="inlineStr">
+        <is>
+          <t>8,35</t>
         </is>
       </c>
       <c r="I75" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>70,771</t>
         </is>
       </c>
       <c r="J75" s="4" t="inlineStr">
@@ -4724,7 +4724,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>CAIXA CAPITAL PROTEGIDO CÍCLICO III FIC FIF MM LP - RESP LTDA (1)</t>
+          <t>CAIXA CAPITAL PROTEGIDO CÍCLICO III FIC FIF MM LP - RESP LTDA</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -4734,32 +4734,32 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E76" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,53337400</t>
+        </is>
+      </c>
+      <c r="E76" s="7" t="inlineStr">
+        <is>
+          <t>-0,004</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G76" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H76" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>0,00</t>
+        </is>
+      </c>
+      <c r="G76" s="3" t="inlineStr">
+        <is>
+          <t>2,69</t>
+        </is>
+      </c>
+      <c r="H76" s="3" t="inlineStr">
+        <is>
+          <t>18,93</t>
         </is>
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14,513</t>
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr">
@@ -4781,7 +4781,7 @@
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>CAIXA CAPITAL PROTEGIDO IBOVESPA CÍCLICO I FIC FIF MM (1)</t>
+          <t>CAIXA CAPITAL PROTEGIDO IBOVESPA CÍCLICO I FIC FIF MM</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
@@ -4791,32 +4791,32 @@
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E77" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F77" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G77" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H77" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>3,25598300</t>
+        </is>
+      </c>
+      <c r="E77" s="6" t="inlineStr">
+        <is>
+          <t>-0,005</t>
+        </is>
+      </c>
+      <c r="F77" s="5" t="inlineStr">
+        <is>
+          <t>1,19</t>
+        </is>
+      </c>
+      <c r="G77" s="5" t="inlineStr">
+        <is>
+          <t>2,19</t>
+        </is>
+      </c>
+      <c r="H77" s="5" t="inlineStr">
+        <is>
+          <t>7,05</t>
         </is>
       </c>
       <c r="I77" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>155,146</t>
         </is>
       </c>
       <c r="J77" s="4" t="inlineStr">
@@ -4838,7 +4838,7 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIM CAPITAL PROTEGIDO CICLICO II LP - RL (1)</t>
+          <t>CAIXA FIC FIM CAPITAL PROTEGIDO CICLICO II LP - RL</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
@@ -4848,32 +4848,32 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E78" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F78" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G78" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H78" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,47220000</t>
+        </is>
+      </c>
+      <c r="E78" s="7" t="inlineStr">
+        <is>
+          <t>-0,003</t>
+        </is>
+      </c>
+      <c r="F78" s="3" t="inlineStr">
+        <is>
+          <t>1,51</t>
+        </is>
+      </c>
+      <c r="G78" s="3" t="inlineStr">
+        <is>
+          <t>1,80</t>
+        </is>
+      </c>
+      <c r="H78" s="3" t="inlineStr">
+        <is>
+          <t>14,37</t>
         </is>
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>190,975</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr">
@@ -4891,7 +4891,7 @@
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF EXPERT PIMCO INCOME IE MM LP RESP LTDA (1)</t>
+          <t>CAIXA FIC FIF EXPERT PIMCO INCOME IE MM LP RESP LTDA</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
@@ -4901,32 +4901,32 @@
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E79" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F79" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G79" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H79" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,41230600</t>
+        </is>
+      </c>
+      <c r="E79" s="6" t="inlineStr">
+        <is>
+          <t>-0,003</t>
+        </is>
+      </c>
+      <c r="F79" s="5" t="inlineStr">
+        <is>
+          <t>0,27</t>
+        </is>
+      </c>
+      <c r="G79" s="5" t="inlineStr">
+        <is>
+          <t>2,51</t>
+        </is>
+      </c>
+      <c r="H79" s="5" t="inlineStr">
+        <is>
+          <t>16,08</t>
         </is>
       </c>
       <c r="I79" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>279,219</t>
         </is>
       </c>
       <c r="J79" s="4" t="inlineStr">
@@ -4948,7 +4948,7 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>CAIXA EXPERT GIANT ZARATHUSTRA FIC MULTIMERCADO - RESP LTDA (1)</t>
+          <t>CAIXA EXPERT GIANT ZARATHUSTRA FIC MULTIMERCADO - RESP LTDA</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
@@ -4958,32 +4958,32 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E80" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F80" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G80" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H80" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,31674000</t>
+        </is>
+      </c>
+      <c r="E80" s="7" t="inlineStr">
+        <is>
+          <t>-0,001</t>
+        </is>
+      </c>
+      <c r="F80" s="3" t="inlineStr">
+        <is>
+          <t>0,57</t>
+        </is>
+      </c>
+      <c r="G80" s="3" t="inlineStr">
+        <is>
+          <t>2,59</t>
+        </is>
+      </c>
+      <c r="H80" s="3" t="inlineStr">
+        <is>
+          <t>2,78</t>
         </is>
       </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13,395</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr">
@@ -5040,7 +5040,7 @@
       </c>
       <c r="I81" s="4" t="inlineStr">
         <is>
-          <t>898,185</t>
+          <t>898,178</t>
         </is>
       </c>
       <c r="J81" s="4" t="inlineStr">
@@ -5097,7 +5097,7 @@
       </c>
       <c r="I82" s="2" t="inlineStr">
         <is>
-          <t>748,991</t>
+          <t>748,992</t>
         </is>
       </c>
       <c r="J82" s="2" t="inlineStr">
@@ -5119,7 +5119,7 @@
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>FIC FIF CAIXA EXPERT BTG PACTUAL X10 MM LP RESP LTDA (1)</t>
+          <t>FIC FIF CAIXA EXPERT BTG PACTUAL X10 MM LP RESP LTDA</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
@@ -5129,32 +5129,32 @@
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E83" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F83" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G83" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H83" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>6,78432500</t>
+        </is>
+      </c>
+      <c r="E83" s="6" t="inlineStr">
+        <is>
+          <t>-0,004</t>
+        </is>
+      </c>
+      <c r="F83" s="5" t="inlineStr">
+        <is>
+          <t>0,09</t>
+        </is>
+      </c>
+      <c r="G83" s="5" t="inlineStr">
+        <is>
+          <t>5,48</t>
+        </is>
+      </c>
+      <c r="H83" s="5" t="inlineStr">
+        <is>
+          <t>16,73</t>
         </is>
       </c>
       <c r="I83" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>129,587</t>
         </is>
       </c>
       <c r="J83" s="4" t="inlineStr">
@@ -5176,7 +5176,7 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF EXPERT SPX NIMITZ MULTIMERCADO RESP LTDA (1)</t>
+          <t>CAIXA FIC FIF EXPERT SPX NIMITZ MULTIMERCADO RESP LTDA</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
@@ -5186,32 +5186,32 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E84" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F84" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G84" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H84" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,77206600</t>
+        </is>
+      </c>
+      <c r="E84" s="7" t="inlineStr">
+        <is>
+          <t>-0,002</t>
+        </is>
+      </c>
+      <c r="F84" s="3" t="inlineStr">
+        <is>
+          <t>0,72</t>
+        </is>
+      </c>
+      <c r="G84" s="3" t="inlineStr">
+        <is>
+          <t>0,31</t>
+        </is>
+      </c>
+      <c r="H84" s="3" t="inlineStr">
+        <is>
+          <t>10,69</t>
         </is>
       </c>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>176,392</t>
         </is>
       </c>
       <c r="J84" s="2" t="inlineStr">
@@ -5268,7 +5268,7 @@
       </c>
       <c r="I85" s="4" t="inlineStr">
         <is>
-          <t>97,614</t>
+          <t>97,597</t>
         </is>
       </c>
       <c r="J85" s="4" t="inlineStr">
@@ -5325,7 +5325,7 @@
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>347,120</t>
+          <t>347,118</t>
         </is>
       </c>
       <c r="J86" s="2" t="inlineStr">
@@ -5439,7 +5439,7 @@
       </c>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t>10,318</t>
+          <t>10,316</t>
         </is>
       </c>
       <c r="J88" s="2" t="inlineStr">
@@ -5492,7 +5492,7 @@
       </c>
       <c r="I89" s="4" t="inlineStr">
         <is>
-          <t>277,722</t>
+          <t>277,543</t>
         </is>
       </c>
       <c r="J89" s="4" t="inlineStr">
@@ -5549,7 +5549,7 @@
       </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>445,938</t>
+          <t>445,937</t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr">
@@ -5606,7 +5606,7 @@
       </c>
       <c r="I91" s="4" t="inlineStr">
         <is>
-          <t>58,253</t>
+          <t>58,191</t>
         </is>
       </c>
       <c r="J91" s="4" t="inlineStr">
@@ -5777,7 +5777,7 @@
       </c>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t>92,434</t>
+          <t>92,431</t>
         </is>
       </c>
       <c r="J94" s="2" t="inlineStr">
@@ -5799,7 +5799,7 @@
       </c>
       <c r="B95" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF AÇÕES MULTIGESTOR RESP LTDA (1)</t>
+          <t>CAIXA FIC FIF AÇÕES MULTIGESTOR RESP LTDA</t>
         </is>
       </c>
       <c r="C95" s="4" t="inlineStr">
@@ -5809,32 +5809,32 @@
       </c>
       <c r="D95" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E95" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F95" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G95" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H95" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1,30185000</t>
+        </is>
+      </c>
+      <c r="E95" s="6" t="inlineStr">
+        <is>
+          <t>-0,024</t>
+        </is>
+      </c>
+      <c r="F95" s="6" t="inlineStr">
+        <is>
+          <t>-4,66</t>
+        </is>
+      </c>
+      <c r="G95" s="5" t="inlineStr">
+        <is>
+          <t>1,14</t>
+        </is>
+      </c>
+      <c r="H95" s="5" t="inlineStr">
+        <is>
+          <t>10,89</t>
         </is>
       </c>
       <c r="I95" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>295,634</t>
         </is>
       </c>
       <c r="J95" s="4" t="inlineStr">
@@ -5891,7 +5891,7 @@
       </c>
       <c r="I96" s="2" t="inlineStr">
         <is>
-          <t>114,110</t>
+          <t>114,109</t>
         </is>
       </c>
       <c r="J96" s="2" t="inlineStr">
@@ -5948,7 +5948,7 @@
       </c>
       <c r="I97" s="4" t="inlineStr">
         <is>
-          <t>133,544</t>
+          <t>133,454</t>
         </is>
       </c>
       <c r="J97" s="4" t="inlineStr">
@@ -6005,7 +6005,7 @@
       </c>
       <c r="I98" s="2" t="inlineStr">
         <is>
-          <t>47,674</t>
+          <t>47,639</t>
         </is>
       </c>
       <c r="J98" s="2" t="inlineStr">
@@ -6058,7 +6058,7 @@
       </c>
       <c r="I99" s="4" t="inlineStr">
         <is>
-          <t>129,900</t>
+          <t>129,793</t>
         </is>
       </c>
       <c r="J99" s="4" t="inlineStr">
@@ -6115,7 +6115,7 @@
       </c>
       <c r="I100" s="2" t="inlineStr">
         <is>
-          <t>41,489</t>
+          <t>41,414</t>
         </is>
       </c>
       <c r="J100" s="2" t="inlineStr">
@@ -6172,7 +6172,7 @@
       </c>
       <c r="I101" s="4" t="inlineStr">
         <is>
-          <t>677,490</t>
+          <t>677,323</t>
         </is>
       </c>
       <c r="J101" s="4" t="inlineStr">
@@ -6229,7 +6229,7 @@
       </c>
       <c r="I102" s="2" t="inlineStr">
         <is>
-          <t>440,323</t>
+          <t>440,272</t>
         </is>
       </c>
       <c r="J102" s="2" t="inlineStr">
@@ -6343,7 +6343,7 @@
       </c>
       <c r="I104" s="2" t="inlineStr">
         <is>
-          <t>30,199</t>
+          <t>30,188</t>
         </is>
       </c>
       <c r="J104" s="2" t="inlineStr">
@@ -6400,7 +6400,7 @@
       </c>
       <c r="I105" s="4" t="inlineStr">
         <is>
-          <t>1,793</t>
+          <t>1,792</t>
         </is>
       </c>
       <c r="J105" s="4" t="inlineStr">
@@ -6457,7 +6457,7 @@
       </c>
       <c r="I106" s="2" t="inlineStr">
         <is>
-          <t>44,434</t>
+          <t>44,404</t>
         </is>
       </c>
       <c r="J106" s="2" t="inlineStr">
@@ -6514,7 +6514,7 @@
       </c>
       <c r="I107" s="4" t="inlineStr">
         <is>
-          <t>36,469</t>
+          <t>36,461</t>
         </is>
       </c>
       <c r="J107" s="4" t="inlineStr">
@@ -6571,7 +6571,7 @@
       </c>
       <c r="I108" s="2" t="inlineStr">
         <is>
-          <t>910,760</t>
+          <t>910,317</t>
         </is>
       </c>
       <c r="J108" s="2" t="inlineStr">
@@ -6628,7 +6628,7 @@
       </c>
       <c r="I109" s="4" t="inlineStr">
         <is>
-          <t>2,994</t>
+          <t>2,993</t>
         </is>
       </c>
       <c r="J109" s="4" t="inlineStr">
@@ -6742,7 +6742,7 @@
       </c>
       <c r="I111" s="4" t="inlineStr">
         <is>
-          <t>19,765</t>
+          <t>19,390</t>
         </is>
       </c>
       <c r="J111" s="4" t="inlineStr">
@@ -6799,7 +6799,7 @@
       </c>
       <c r="I112" s="2" t="inlineStr">
         <is>
-          <t>269,776</t>
+          <t>269,513</t>
         </is>
       </c>
       <c r="J112" s="2" t="inlineStr">
@@ -6821,7 +6821,7 @@
       </c>
       <c r="B113" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC ACOES EXPERT VERDE AM LONG BIAS - RESP LTDA (1)</t>
+          <t>CAIXA FIC ACOES EXPERT VERDE AM LONG BIAS - RESP LTDA</t>
         </is>
       </c>
       <c r="C113" s="4" t="inlineStr">
@@ -6831,32 +6831,32 @@
       </c>
       <c r="D113" s="4" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E113" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F113" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G113" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H113" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1.017,29224100</t>
+        </is>
+      </c>
+      <c r="E113" s="6" t="inlineStr">
+        <is>
+          <t>-0,003</t>
+        </is>
+      </c>
+      <c r="F113" s="6" t="inlineStr">
+        <is>
+          <t>-4,92</t>
+        </is>
+      </c>
+      <c r="G113" s="5" t="inlineStr">
+        <is>
+          <t>3,76</t>
+        </is>
+      </c>
+      <c r="H113" s="5" t="inlineStr">
+        <is>
+          <t>19,30</t>
         </is>
       </c>
       <c r="I113" s="4" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>8,171</t>
         </is>
       </c>
       <c r="J113" s="4" t="inlineStr">
@@ -6878,7 +6878,7 @@
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>CAIXA EXPERT CLARITAS VALOR FIC FIF AÇÕES - RESP LTDA (1)</t>
+          <t>CAIXA EXPERT CLARITAS VALOR FIC FIF AÇÕES - RESP LTDA</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
@@ -6888,32 +6888,32 @@
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E114" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F114" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G114" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H114" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>1.538,75924600</t>
+        </is>
+      </c>
+      <c r="E114" s="7" t="inlineStr">
+        <is>
+          <t>-0,002</t>
+        </is>
+      </c>
+      <c r="F114" s="7" t="inlineStr">
+        <is>
+          <t>-4,34</t>
+        </is>
+      </c>
+      <c r="G114" s="3" t="inlineStr">
+        <is>
+          <t>2,87</t>
+        </is>
+      </c>
+      <c r="H114" s="3" t="inlineStr">
+        <is>
+          <t>15,06</t>
         </is>
       </c>
       <c r="I114" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>22,409</t>
         </is>
       </c>
       <c r="J114" s="2" t="inlineStr">
@@ -6945,7 +6945,7 @@
       </c>
       <c r="D115" s="4" t="inlineStr">
         <is>
-          <t>172,97549800</t>
+          <t>172,97549798</t>
         </is>
       </c>
       <c r="E115" s="6" t="inlineStr">
@@ -7080,7 +7080,7 @@
       </c>
       <c r="I117" s="4" t="inlineStr">
         <is>
-          <t>1.692,073</t>
+          <t>1.691,330</t>
         </is>
       </c>
       <c r="J117" s="4" t="inlineStr">
@@ -7133,7 +7133,7 @@
       </c>
       <c r="I118" s="2" t="inlineStr">
         <is>
-          <t>730,865</t>
+          <t>730,347</t>
         </is>
       </c>
       <c r="J118" s="2" t="inlineStr">
@@ -7186,7 +7186,7 @@
       </c>
       <c r="I119" s="4" t="inlineStr">
         <is>
-          <t>797,168</t>
+          <t>796,676</t>
         </is>
       </c>
       <c r="J119" s="4" t="inlineStr">
@@ -7345,7 +7345,7 @@
       </c>
       <c r="I122" s="2" t="inlineStr">
         <is>
-          <t>633,334</t>
+          <t>632,633</t>
         </is>
       </c>
       <c r="J122" s="2" t="inlineStr">
@@ -7398,7 +7398,7 @@
       </c>
       <c r="I123" s="4" t="inlineStr">
         <is>
-          <t>477,359</t>
+          <t>476,930</t>
         </is>
       </c>
       <c r="J123" s="4" t="inlineStr">
@@ -7451,7 +7451,7 @@
       </c>
       <c r="I124" s="2" t="inlineStr">
         <is>
-          <t>728,420</t>
+          <t>727,765</t>
         </is>
       </c>
       <c r="J124" s="2" t="inlineStr">
@@ -7469,7 +7469,7 @@
       </c>
       <c r="B125" s="4" t="inlineStr">
         <is>
-          <t>CAIXA AZULZINHA FIC FIF RF SIMPLES - RESP LTDA (2)</t>
+          <t>CAIXA AZULZINHA FIC FIF RF SIMPLES - RESP LTDA (2) (8)</t>
         </is>
       </c>
       <c r="C125" s="4" t="inlineStr">
@@ -7526,7 +7526,7 @@
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF AMETISTA CORP RF SIMPLES RESP LTDA</t>
+          <t>CAIXA FIC FIF AMETISTA CORP RF SIMPLES RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C126" s="2" t="inlineStr">
@@ -7561,7 +7561,7 @@
       </c>
       <c r="I126" s="2" t="inlineStr">
         <is>
-          <t>278,896</t>
+          <t>210,583</t>
         </is>
       </c>
       <c r="J126" s="2" t="inlineStr">
@@ -7618,7 +7618,7 @@
       </c>
       <c r="I127" s="4" t="inlineStr">
         <is>
-          <t>41,349</t>
+          <t>41,348</t>
         </is>
       </c>
       <c r="J127" s="4" t="inlineStr">
@@ -7846,7 +7846,7 @@
       </c>
       <c r="I131" s="4" t="inlineStr">
         <is>
-          <t>7.911,086</t>
+          <t>7.746,819</t>
         </is>
       </c>
       <c r="J131" s="4" t="inlineStr">
@@ -7903,7 +7903,7 @@
       </c>
       <c r="I132" s="2" t="inlineStr">
         <is>
-          <t>15.188,951</t>
+          <t>15.188,427</t>
         </is>
       </c>
       <c r="J132" s="2" t="inlineStr">
@@ -7960,7 +7960,7 @@
       </c>
       <c r="I133" s="4" t="inlineStr">
         <is>
-          <t>3.102,003</t>
+          <t>3.101,995</t>
         </is>
       </c>
       <c r="J133" s="4" t="inlineStr">
@@ -7982,7 +7982,7 @@
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC INST SOBERANO PLUS RF</t>
+          <t>CAIXA FIC INST SOBERANO PLUS RF (8)</t>
         </is>
       </c>
       <c r="C134" s="2" t="inlineStr">
@@ -7992,7 +7992,7 @@
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>1,53832400</t>
+          <t>1,53832366</t>
         </is>
       </c>
       <c r="E134" s="3" t="inlineStr">
@@ -8017,7 +8017,7 @@
       </c>
       <c r="I134" s="2" t="inlineStr">
         <is>
-          <t>351,682</t>
+          <t>349,182</t>
         </is>
       </c>
       <c r="J134" s="2" t="inlineStr">
@@ -8245,7 +8245,7 @@
       </c>
       <c r="I138" s="2" t="inlineStr">
         <is>
-          <t>13.630,096</t>
+          <t>13.358,530</t>
         </is>
       </c>
       <c r="J138" s="2" t="inlineStr">
@@ -8302,7 +8302,7 @@
       </c>
       <c r="I139" s="4" t="inlineStr">
         <is>
-          <t>12.332,869</t>
+          <t>12.332,337</t>
         </is>
       </c>
       <c r="J139" s="4" t="inlineStr">
@@ -8359,7 +8359,7 @@
       </c>
       <c r="I140" s="2" t="inlineStr">
         <is>
-          <t>3.760,319</t>
+          <t>3.760,105</t>
         </is>
       </c>
       <c r="J140" s="2" t="inlineStr">
@@ -8381,7 +8381,7 @@
       </c>
       <c r="B141" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF TURQUESA CORPORATIVO RF CP RESP LTDA</t>
+          <t>CAIXA FIC FIF TURQUESA CORPORATIVO RF CP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C141" s="4" t="inlineStr">
@@ -8416,7 +8416,7 @@
       </c>
       <c r="I141" s="4" t="inlineStr">
         <is>
-          <t>1.405,753</t>
+          <t>1.405,645</t>
         </is>
       </c>
       <c r="J141" s="4" t="inlineStr">
@@ -8438,7 +8438,7 @@
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF AUTOMATICO POLIS RF CURTO PRAZO RESP LTDA</t>
+          <t>CAIXA FIC FIF AUTOMATICO POLIS RF CURTO PRAZO RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C142" s="2" t="inlineStr">
@@ -8473,7 +8473,7 @@
       </c>
       <c r="I142" s="2" t="inlineStr">
         <is>
-          <t>33.663,684</t>
+          <t>33.436,643</t>
         </is>
       </c>
       <c r="J142" s="2" t="inlineStr">
@@ -8495,7 +8495,7 @@
       </c>
       <c r="B143" s="4" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF PRÁTICO RF CURTO PRAZO RESP LTDA</t>
+          <t>CAIXA FIC FIF PRÁTICO RF CURTO PRAZO RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C143" s="4" t="inlineStr">
@@ -8530,7 +8530,7 @@
       </c>
       <c r="I143" s="4" t="inlineStr">
         <is>
-          <t>2.913,398</t>
+          <t>2.900,764</t>
         </is>
       </c>
       <c r="J143" s="4" t="inlineStr">
@@ -8552,7 +8552,7 @@
       </c>
       <c r="B144" s="2" t="inlineStr">
         <is>
-          <t>CAIXA FIC FIF TRANSFERÊNCIA VOLUNTÁRIA RF CP RESP LTDA</t>
+          <t>CAIXA FIC FIF TRANSFERÊNCIA VOLUNTÁRIA RF CP RESP LTDA (8)</t>
         </is>
       </c>
       <c r="C144" s="2" t="inlineStr">
@@ -8587,7 +8587,7 @@
       </c>
       <c r="I144" s="2" t="inlineStr">
         <is>
-          <t>14.478,393</t>
+          <t>14.686,376</t>
         </is>
       </c>
       <c r="J144" s="2" t="inlineStr">
@@ -8644,7 +8644,7 @@
       </c>
       <c r="I145" s="4" t="inlineStr">
         <is>
-          <t>9.177,241</t>
+          <t>9.177,239</t>
         </is>
       </c>
       <c r="J145" s="4" t="inlineStr">
@@ -9385,7 +9385,7 @@
       </c>
       <c r="I158" s="2" t="inlineStr">
         <is>
-          <t>13.071,443</t>
+          <t>13.071,442</t>
         </is>
       </c>
       <c r="J158" s="2" t="inlineStr">
@@ -9556,7 +9556,7 @@
       </c>
       <c r="I161" s="4" t="inlineStr">
         <is>
-          <t>1.554,634</t>
+          <t>1.645,842</t>
         </is>
       </c>
       <c r="J161" s="4" t="inlineStr">
@@ -9613,7 +9613,7 @@
       </c>
       <c r="I162" s="2" t="inlineStr">
         <is>
-          <t>24.730,802</t>
+          <t>24.730,801</t>
         </is>
       </c>
       <c r="J162" s="2" t="inlineStr">
@@ -9784,7 +9784,7 @@
       </c>
       <c r="I165" s="4" t="inlineStr">
         <is>
-          <t>301,178</t>
+          <t>301,175</t>
         </is>
       </c>
       <c r="J165" s="4" t="inlineStr">
@@ -9873,7 +9873,7 @@
       </c>
       <c r="D167" s="4" t="inlineStr">
         <is>
-          <t>11,26019000</t>
+          <t>11,26018960</t>
         </is>
       </c>
       <c r="E167" s="5" t="inlineStr">
@@ -10040,7 +10040,7 @@
       </c>
       <c r="D170" s="2" t="inlineStr">
         <is>
-          <t>3,47467000</t>
+          <t>3,47467001</t>
         </is>
       </c>
       <c r="E170" s="7" t="inlineStr">
@@ -10097,7 +10097,7 @@
       </c>
       <c r="D171" s="4" t="inlineStr">
         <is>
-          <t>2,54576900</t>
+          <t>2,54576924</t>
         </is>
       </c>
       <c r="E171" s="6" t="inlineStr">
@@ -10179,7 +10179,7 @@
       </c>
       <c r="I172" s="2" t="inlineStr">
         <is>
-          <t>4.941,247</t>
+          <t>4.940,924</t>
         </is>
       </c>
       <c r="J172" s="2" t="inlineStr">

</xml_diff>